<commit_message>
econ: self-healing price recalc + honest annual savings
</commit_message>
<xml_diff>
--- a/data/raw/prices_wb.xlsx
+++ b/data/raw/prices_wb.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I160"/>
+  <dimension ref="A1:I169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6438,21 +6438,21 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>OVER Глицин + Гинкго Билоба + Готу Кола, 60 капсул</t>
+          <t>Alantra Готу Кола капсулы Алантра, 500 мг*60 шт</t>
         </is>
       </c>
       <c r="C155" t="n">
         <v>60</v>
       </c>
       <c r="D155" t="n">
-        <v>674</v>
+        <v>961</v>
       </c>
       <c r="E155" t="n">
         <v>30</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>WB арт.167807321</t>
+          <t>WB арт.978377015</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -6461,11 +6461,11 @@
         </is>
       </c>
       <c r="H155" t="n">
-        <v>337</v>
+        <v>480</v>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>средний</t>
+          <t>премиум</t>
         </is>
       </c>
     </row>
@@ -6477,21 +6477,21 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Alantra Готу Кола капсулы Алантра, 500 мг*60 шт</t>
+          <t>NOW Gotu Kola Готу Кола, Центелла Азиатская 450 мг - 100 капсул</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D156" t="n">
-        <v>961</v>
+        <v>1046</v>
       </c>
       <c r="E156" t="n">
         <v>30</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>WB арт.978377015</t>
+          <t>WB арт.138748103</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -6500,11 +6500,11 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>480</v>
+        <v>314</v>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>премиум</t>
+          <t>эконом</t>
         </is>
       </c>
     </row>
@@ -6516,21 +6516,21 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>NOW Gotu Kola Готу Кола, Центелла Азиатская 450 мг - 100 капсул</t>
+          <t>Nature's way Готу Кола 100 капсул</t>
         </is>
       </c>
       <c r="C157" t="n">
         <v>100</v>
       </c>
       <c r="D157" t="n">
-        <v>1046</v>
+        <v>2455</v>
       </c>
       <c r="E157" t="n">
         <v>30</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>WB арт.138748103</t>
+          <t>WB арт.447867459</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -6539,11 +6539,11 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>314</v>
+        <v>736</v>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>эконом</t>
+          <t>премиум</t>
         </is>
       </c>
     </row>
@@ -6555,21 +6555,21 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Nature's way Готу Кола 100 капсул</t>
+          <t>Shri Ganga Для памяти и улучшения слуха Гото Кула Goto Kula 100 таб</t>
         </is>
       </c>
       <c r="C158" t="n">
         <v>100</v>
       </c>
       <c r="D158" t="n">
-        <v>2455</v>
+        <v>473</v>
       </c>
       <c r="E158" t="n">
         <v>30</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>WB арт.447867459</t>
+          <t>WB арт.924661260</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -6578,11 +6578,11 @@
         </is>
       </c>
       <c r="H158" t="n">
-        <v>736</v>
+        <v>142</v>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>премиум</t>
+          <t>эконом</t>
         </is>
       </c>
     </row>
@@ -6594,21 +6594,21 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Shri Ganga Для памяти и улучшения слуха Гото Кула Goto Kula 100 таб</t>
+          <t>GLS pharmaceuticals Гинкго билоба+Готу кола GLS капсулы по 380 мг 60 шт</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D159" t="n">
-        <v>473</v>
+        <v>727</v>
       </c>
       <c r="E159" t="n">
         <v>30</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>WB арт.924661260</t>
+          <t>WB арт.822682995</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -6617,37 +6617,37 @@
         </is>
       </c>
       <c r="H159" t="n">
-        <v>142</v>
+        <v>364</v>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>эконом</t>
+          <t>средний</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Готу кола</t>
+          <t>Креатин</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>GLS pharmaceuticals Гинкго билоба+Готу кола GLS капсулы по 380 мг 60 шт</t>
+          <t>Prime Kraft Креатин моногидрат Creatine Monohydrate, без вкуса 200 гр</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="D160" t="n">
-        <v>727</v>
+        <v>640</v>
       </c>
       <c r="E160" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>WB арт.822682995</t>
+          <t>WB арт.4219394</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -6656,13 +6656,324 @@
         </is>
       </c>
       <c r="H160" t="n">
-        <v>364</v>
-      </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>средний</t>
-        </is>
-      </c>
+        <v>480</v>
+      </c>
+      <c r="I160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин Creatine Monohydrate 100% Pure (без вкуса), 500 гр</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>500</v>
+      </c>
+      <c r="D161" t="n">
+        <v>1411</v>
+      </c>
+      <c r="E161" t="n">
+        <v>150</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>WB арт.13257465</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H161" t="n">
+        <v>423</v>
+      </c>
+      <c r="I161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин Creatine Monohydrate, Вишня 200 гр</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>200</v>
+      </c>
+      <c r="D162" t="n">
+        <v>660</v>
+      </c>
+      <c r="E162" t="n">
+        <v>150</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>WB арт.120930475</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H162" t="n">
+        <v>495</v>
+      </c>
+      <c r="I162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин Creatine Monohydrate, Энергетик 200 гр</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>200</v>
+      </c>
+      <c r="D163" t="n">
+        <v>660</v>
+      </c>
+      <c r="E163" t="n">
+        <v>150</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>WB арт.228766204</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H163" t="n">
+        <v>495</v>
+      </c>
+      <c r="I163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин Creatine Monohydrate, Ананас 200 гр</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>200</v>
+      </c>
+      <c r="D164" t="n">
+        <v>845</v>
+      </c>
+      <c r="E164" t="n">
+        <v>150</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>WB арт.120930473</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H164" t="n">
+        <v>634</v>
+      </c>
+      <c r="I164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин Creatine Monohydrate, Цитрусовый микс 200 гр</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>200</v>
+      </c>
+      <c r="D165" t="n">
+        <v>563</v>
+      </c>
+      <c r="E165" t="n">
+        <v>150</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>WB арт.120930474</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H165" t="n">
+        <v>422</v>
+      </c>
+      <c r="I165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин Creatine Monohydrate, Вишня 500 гр</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>500</v>
+      </c>
+      <c r="D166" t="n">
+        <v>1525</v>
+      </c>
+      <c r="E166" t="n">
+        <v>150</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>WB арт.183766036</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H166" t="n">
+        <v>458</v>
+      </c>
+      <c r="I166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин Creatine Monohydrate Pineapple (ананас), 500 гр</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>500</v>
+      </c>
+      <c r="D167" t="n">
+        <v>1490</v>
+      </c>
+      <c r="E167" t="n">
+        <v>150</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>WB арт.183766034</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H167" t="n">
+        <v>447</v>
+      </c>
+      <c r="I167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>BIOVIN Креатин моногидрат порошок, спортивное питание creatine 300г</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>300</v>
+      </c>
+      <c r="D168" t="n">
+        <v>385</v>
+      </c>
+      <c r="E168" t="n">
+        <v>150</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>WB арт.59102656</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H168" t="n">
+        <v>193</v>
+      </c>
+      <c r="I168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Креатин</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Prime Kraft Креатин моногидрат микронизированный, фруктовый пунш 200 гр</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>200</v>
+      </c>
+      <c r="D169" t="n">
+        <v>668</v>
+      </c>
+      <c r="E169" t="n">
+        <v>150</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>WB арт.213577274</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="H169" t="n">
+        <v>501</v>
+      </c>
+      <c r="I169" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
viz: final chart set (waterfall, heatmap, bubble) - clean data
</commit_message>
<xml_diff>
--- a/data/raw/prices_wb.xlsx
+++ b/data/raw/prices_wb.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\analytics\brain-25-evidence\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D7D3F5-06F5-4300-8D78-10B5CD42AD6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C446CF9-8270-4A34-8C70-AB5318F4B949}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="364">
   <si>
     <t>добавка</t>
   </si>
@@ -467,12 +467,6 @@
   </si>
   <si>
     <t>WB арт.822680108</t>
-  </si>
-  <si>
-    <t>– Родиолы экстракт жидкий для приема внутрь 30 мл 1 шт</t>
-  </si>
-  <si>
-    <t>WB арт.822684736</t>
   </si>
   <si>
     <t>эколаб Родиола + витамин С 90 капсул</t>
@@ -1457,7 +1451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I168"/>
+  <dimension ref="A1:I167"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3324,10 +3318,10 @@
         <v>149</v>
       </c>
       <c r="C65">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="D65">
-        <v>140</v>
+        <v>604</v>
       </c>
       <c r="E65">
         <v>30</v>
@@ -3339,36 +3333,36 @@
         <v>12</v>
       </c>
       <c r="H65">
-        <v>4200</v>
+        <v>201</v>
       </c>
       <c r="I65" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B66" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C66">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D66">
-        <v>604</v>
+        <v>1839</v>
       </c>
       <c r="E66">
         <v>30</v>
       </c>
       <c r="F66" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G66" t="s">
         <v>12</v>
       </c>
       <c r="H66">
-        <v>201</v>
+        <v>920</v>
       </c>
       <c r="I66" t="s">
         <v>13</v>
@@ -3376,7 +3370,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B67" t="s">
         <v>154</v>
@@ -3385,7 +3379,7 @@
         <v>60</v>
       </c>
       <c r="D67">
-        <v>1839</v>
+        <v>2586</v>
       </c>
       <c r="E67">
         <v>30</v>
@@ -3397,15 +3391,15 @@
         <v>12</v>
       </c>
       <c r="H67">
-        <v>920</v>
+        <v>1293</v>
       </c>
       <c r="I67" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B68" t="s">
         <v>156</v>
@@ -3414,7 +3408,7 @@
         <v>60</v>
       </c>
       <c r="D68">
-        <v>2586</v>
+        <v>2799</v>
       </c>
       <c r="E68">
         <v>30</v>
@@ -3426,7 +3420,7 @@
         <v>12</v>
       </c>
       <c r="H68">
-        <v>1293</v>
+        <v>1400</v>
       </c>
       <c r="I68" t="s">
         <v>16</v>
@@ -3434,16 +3428,16 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B69" t="s">
         <v>158</v>
       </c>
       <c r="C69">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D69">
-        <v>2799</v>
+        <v>1994</v>
       </c>
       <c r="E69">
         <v>30</v>
@@ -3455,24 +3449,24 @@
         <v>12</v>
       </c>
       <c r="H69">
-        <v>1400</v>
+        <v>1994</v>
       </c>
       <c r="I69" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B70" t="s">
         <v>160</v>
       </c>
       <c r="C70">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D70">
-        <v>1994</v>
+        <v>4198</v>
       </c>
       <c r="E70">
         <v>30</v>
@@ -3484,7 +3478,7 @@
         <v>12</v>
       </c>
       <c r="H70">
-        <v>1994</v>
+        <v>2099</v>
       </c>
       <c r="I70" t="s">
         <v>19</v>
@@ -3492,16 +3486,16 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B71" t="s">
         <v>162</v>
       </c>
       <c r="C71">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D71">
-        <v>4198</v>
+        <v>4654</v>
       </c>
       <c r="E71">
         <v>30</v>
@@ -3513,24 +3507,24 @@
         <v>12</v>
       </c>
       <c r="H71">
-        <v>2099</v>
+        <v>1164</v>
       </c>
       <c r="I71" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B72" t="s">
         <v>164</v>
       </c>
       <c r="C72">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D72">
-        <v>4654</v>
+        <v>4365</v>
       </c>
       <c r="E72">
         <v>30</v>
@@ -3542,24 +3536,24 @@
         <v>12</v>
       </c>
       <c r="H72">
-        <v>1164</v>
+        <v>2182</v>
       </c>
       <c r="I72" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B73" t="s">
         <v>166</v>
       </c>
       <c r="C73">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D73">
-        <v>4365</v>
+        <v>2799</v>
       </c>
       <c r="E73">
         <v>30</v>
@@ -3571,53 +3565,53 @@
         <v>12</v>
       </c>
       <c r="H73">
-        <v>2182</v>
+        <v>700</v>
       </c>
       <c r="I73" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="B74" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C74">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D74">
-        <v>2799</v>
+        <v>2818</v>
       </c>
       <c r="E74">
         <v>30</v>
       </c>
       <c r="F74" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G74" t="s">
         <v>12</v>
       </c>
       <c r="H74">
-        <v>700</v>
+        <v>1409</v>
       </c>
       <c r="I74" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B75" t="s">
         <v>171</v>
       </c>
       <c r="C75">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="D75">
-        <v>2818</v>
+        <v>3868</v>
       </c>
       <c r="E75">
         <v>30</v>
@@ -3629,24 +3623,24 @@
         <v>12</v>
       </c>
       <c r="H75">
-        <v>1409</v>
+        <v>1289</v>
       </c>
       <c r="I75" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B76" t="s">
         <v>173</v>
       </c>
       <c r="C76">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D76">
-        <v>3868</v>
+        <v>3498</v>
       </c>
       <c r="E76">
         <v>30</v>
@@ -3658,15 +3652,15 @@
         <v>12</v>
       </c>
       <c r="H76">
-        <v>1289</v>
+        <v>1749</v>
       </c>
       <c r="I76" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B77" t="s">
         <v>175</v>
@@ -3675,7 +3669,7 @@
         <v>60</v>
       </c>
       <c r="D77">
-        <v>3498</v>
+        <v>1517</v>
       </c>
       <c r="E77">
         <v>30</v>
@@ -3687,15 +3681,15 @@
         <v>12</v>
       </c>
       <c r="H77">
-        <v>1749</v>
+        <v>758</v>
       </c>
       <c r="I77" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B78" t="s">
         <v>177</v>
@@ -3704,7 +3698,7 @@
         <v>60</v>
       </c>
       <c r="D78">
-        <v>1517</v>
+        <v>2970</v>
       </c>
       <c r="E78">
         <v>30</v>
@@ -3716,15 +3710,15 @@
         <v>12</v>
       </c>
       <c r="H78">
-        <v>758</v>
+        <v>1485</v>
       </c>
       <c r="I78" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B79" t="s">
         <v>179</v>
@@ -3733,7 +3727,7 @@
         <v>60</v>
       </c>
       <c r="D79">
-        <v>2970</v>
+        <v>1584</v>
       </c>
       <c r="E79">
         <v>30</v>
@@ -3745,24 +3739,24 @@
         <v>12</v>
       </c>
       <c r="H79">
-        <v>1485</v>
+        <v>792</v>
       </c>
       <c r="I79" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B80" t="s">
         <v>181</v>
       </c>
       <c r="C80">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="D80">
-        <v>1584</v>
+        <v>3947</v>
       </c>
       <c r="E80">
         <v>30</v>
@@ -3774,53 +3768,53 @@
         <v>12</v>
       </c>
       <c r="H80">
-        <v>792</v>
+        <v>1316</v>
       </c>
       <c r="I80" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="B81" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C81">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="D81">
-        <v>3947</v>
+        <v>1824</v>
       </c>
       <c r="E81">
         <v>30</v>
       </c>
       <c r="F81" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G81" t="s">
         <v>12</v>
       </c>
       <c r="H81">
-        <v>1316</v>
+        <v>5472</v>
       </c>
       <c r="I81" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B82" t="s">
         <v>186</v>
       </c>
       <c r="C82">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D82">
-        <v>1824</v>
+        <v>271</v>
       </c>
       <c r="E82">
         <v>30</v>
@@ -3832,24 +3826,24 @@
         <v>12</v>
       </c>
       <c r="H82">
-        <v>5472</v>
+        <v>1626</v>
       </c>
       <c r="I82" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B83" t="s">
         <v>188</v>
       </c>
       <c r="C83">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="D83">
-        <v>271</v>
+        <v>3714</v>
       </c>
       <c r="E83">
         <v>30</v>
@@ -3861,44 +3855,44 @@
         <v>12</v>
       </c>
       <c r="H83">
-        <v>1626</v>
+        <v>1857</v>
       </c>
       <c r="I83" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B84" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C84">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D84">
-        <v>3714</v>
+        <v>3667</v>
       </c>
       <c r="E84">
         <v>30</v>
       </c>
       <c r="F84" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G84" t="s">
         <v>12</v>
       </c>
       <c r="H84">
-        <v>1857</v>
+        <v>917</v>
       </c>
       <c r="I84" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B85" t="s">
         <v>193</v>
@@ -3907,7 +3901,7 @@
         <v>120</v>
       </c>
       <c r="D85">
-        <v>3667</v>
+        <v>3949</v>
       </c>
       <c r="E85">
         <v>30</v>
@@ -3919,24 +3913,24 @@
         <v>12</v>
       </c>
       <c r="H85">
-        <v>917</v>
+        <v>987</v>
       </c>
       <c r="I85" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B86" t="s">
         <v>195</v>
       </c>
       <c r="C86">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="D86">
-        <v>3949</v>
+        <v>11280</v>
       </c>
       <c r="E86">
         <v>30</v>
@@ -3948,24 +3942,24 @@
         <v>12</v>
       </c>
       <c r="H86">
-        <v>987</v>
+        <v>1410</v>
       </c>
       <c r="I86" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B87" t="s">
         <v>197</v>
       </c>
       <c r="C87">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="D87">
-        <v>11280</v>
+        <v>4229</v>
       </c>
       <c r="E87">
         <v>30</v>
@@ -3977,7 +3971,7 @@
         <v>12</v>
       </c>
       <c r="H87">
-        <v>1410</v>
+        <v>1057</v>
       </c>
       <c r="I87" t="s">
         <v>19</v>
@@ -3985,16 +3979,16 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B88" t="s">
         <v>199</v>
       </c>
       <c r="C88">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="D88">
-        <v>4229</v>
+        <v>4088</v>
       </c>
       <c r="E88">
         <v>30</v>
@@ -4006,82 +4000,82 @@
         <v>12</v>
       </c>
       <c r="H88">
-        <v>1057</v>
+        <v>511</v>
       </c>
       <c r="I88" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B89" t="s">
+        <v>197</v>
+      </c>
+      <c r="C89">
+        <v>120</v>
+      </c>
+      <c r="D89">
+        <v>3722</v>
+      </c>
+      <c r="E89">
+        <v>30</v>
+      </c>
+      <c r="F89" t="s">
         <v>201</v>
       </c>
-      <c r="C89">
-        <v>240</v>
-      </c>
-      <c r="D89">
-        <v>4088</v>
-      </c>
-      <c r="E89">
-        <v>30</v>
-      </c>
-      <c r="F89" t="s">
-        <v>202</v>
-      </c>
       <c r="G89" t="s">
         <v>12</v>
       </c>
       <c r="H89">
-        <v>511</v>
+        <v>930</v>
       </c>
       <c r="I89" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B90" t="s">
         <v>199</v>
       </c>
       <c r="C90">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="D90">
-        <v>3722</v>
+        <v>4051</v>
       </c>
       <c r="E90">
         <v>30</v>
       </c>
       <c r="F90" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G90" t="s">
         <v>12</v>
       </c>
       <c r="H90">
-        <v>930</v>
+        <v>506</v>
       </c>
       <c r="I90" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B91" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C91">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="D91">
-        <v>4051</v>
+        <v>2295</v>
       </c>
       <c r="E91">
         <v>30</v>
@@ -4093,36 +4087,36 @@
         <v>12</v>
       </c>
       <c r="H91">
-        <v>506</v>
+        <v>1148</v>
       </c>
       <c r="I91" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="B92" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C92">
         <v>60</v>
       </c>
       <c r="D92">
-        <v>2295</v>
+        <v>1683</v>
       </c>
       <c r="E92">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F92" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G92" t="s">
         <v>12</v>
       </c>
       <c r="H92">
-        <v>1148</v>
+        <v>1683</v>
       </c>
       <c r="I92" t="s">
         <v>19</v>
@@ -4130,7 +4124,7 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B93" t="s">
         <v>208</v>
@@ -4139,7 +4133,7 @@
         <v>60</v>
       </c>
       <c r="D93">
-        <v>1683</v>
+        <v>467</v>
       </c>
       <c r="E93">
         <v>60</v>
@@ -4151,15 +4145,15 @@
         <v>12</v>
       </c>
       <c r="H93">
-        <v>1683</v>
+        <v>467</v>
       </c>
       <c r="I93" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B94" t="s">
         <v>210</v>
@@ -4168,7 +4162,7 @@
         <v>60</v>
       </c>
       <c r="D94">
-        <v>467</v>
+        <v>342</v>
       </c>
       <c r="E94">
         <v>60</v>
@@ -4180,7 +4174,7 @@
         <v>12</v>
       </c>
       <c r="H94">
-        <v>467</v>
+        <v>342</v>
       </c>
       <c r="I94" t="s">
         <v>13</v>
@@ -4188,7 +4182,7 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B95" t="s">
         <v>212</v>
@@ -4197,7 +4191,7 @@
         <v>60</v>
       </c>
       <c r="D95">
-        <v>342</v>
+        <v>750</v>
       </c>
       <c r="E95">
         <v>60</v>
@@ -4209,24 +4203,24 @@
         <v>12</v>
       </c>
       <c r="H95">
-        <v>342</v>
+        <v>750</v>
       </c>
       <c r="I95" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B96" t="s">
         <v>214</v>
       </c>
       <c r="C96">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D96">
-        <v>750</v>
+        <v>679</v>
       </c>
       <c r="E96">
         <v>60</v>
@@ -4238,24 +4232,24 @@
         <v>12</v>
       </c>
       <c r="H96">
-        <v>750</v>
+        <v>340</v>
       </c>
       <c r="I96" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B97" t="s">
         <v>216</v>
       </c>
       <c r="C97">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="D97">
-        <v>679</v>
+        <v>2553</v>
       </c>
       <c r="E97">
         <v>60</v>
@@ -4267,24 +4261,24 @@
         <v>12</v>
       </c>
       <c r="H97">
-        <v>340</v>
+        <v>5106</v>
       </c>
       <c r="I97" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B98" t="s">
         <v>218</v>
       </c>
       <c r="C98">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D98">
-        <v>2553</v>
+        <v>820</v>
       </c>
       <c r="E98">
         <v>60</v>
@@ -4296,24 +4290,24 @@
         <v>12</v>
       </c>
       <c r="H98">
-        <v>5106</v>
+        <v>820</v>
       </c>
       <c r="I98" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B99" t="s">
         <v>220</v>
       </c>
       <c r="C99">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D99">
-        <v>820</v>
+        <v>681</v>
       </c>
       <c r="E99">
         <v>60</v>
@@ -4325,15 +4319,15 @@
         <v>12</v>
       </c>
       <c r="H99">
-        <v>820</v>
+        <v>1362</v>
       </c>
       <c r="I99" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B100" t="s">
         <v>222</v>
@@ -4342,7 +4336,7 @@
         <v>30</v>
       </c>
       <c r="D100">
-        <v>681</v>
+        <v>606</v>
       </c>
       <c r="E100">
         <v>60</v>
@@ -4354,44 +4348,44 @@
         <v>12</v>
       </c>
       <c r="H100">
-        <v>1362</v>
+        <v>1212</v>
       </c>
       <c r="I100" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
       <c r="B101" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C101">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D101">
-        <v>606</v>
+        <v>812</v>
       </c>
       <c r="E101">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F101" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G101" t="s">
         <v>12</v>
       </c>
       <c r="H101">
-        <v>1212</v>
+        <v>406</v>
       </c>
       <c r="I101" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B102" t="s">
         <v>227</v>
@@ -4400,7 +4394,7 @@
         <v>60</v>
       </c>
       <c r="D102">
-        <v>812</v>
+        <v>245</v>
       </c>
       <c r="E102">
         <v>30</v>
@@ -4412,7 +4406,7 @@
         <v>12</v>
       </c>
       <c r="H102">
-        <v>406</v>
+        <v>122</v>
       </c>
       <c r="I102" t="s">
         <v>13</v>
@@ -4420,16 +4414,16 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B103" t="s">
         <v>229</v>
       </c>
       <c r="C103">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="D103">
-        <v>245</v>
+        <v>1062</v>
       </c>
       <c r="E103">
         <v>30</v>
@@ -4441,7 +4435,7 @@
         <v>12</v>
       </c>
       <c r="H103">
-        <v>122</v>
+        <v>354</v>
       </c>
       <c r="I103" t="s">
         <v>13</v>
@@ -4449,16 +4443,16 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B104" t="s">
         <v>231</v>
       </c>
       <c r="C104">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D104">
-        <v>1062</v>
+        <v>1584</v>
       </c>
       <c r="E104">
         <v>30</v>
@@ -4470,15 +4464,15 @@
         <v>12</v>
       </c>
       <c r="H104">
-        <v>354</v>
+        <v>792</v>
       </c>
       <c r="I104" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B105" t="s">
         <v>233</v>
@@ -4487,7 +4481,7 @@
         <v>60</v>
       </c>
       <c r="D105">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="E105">
         <v>30</v>
@@ -4507,7 +4501,7 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B106" t="s">
         <v>235</v>
@@ -4516,7 +4510,7 @@
         <v>60</v>
       </c>
       <c r="D106">
-        <v>1585</v>
+        <v>1722</v>
       </c>
       <c r="E106">
         <v>30</v>
@@ -4528,53 +4522,53 @@
         <v>12</v>
       </c>
       <c r="H106">
-        <v>792</v>
+        <v>861</v>
       </c>
       <c r="I106" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="B107" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C107">
         <v>60</v>
       </c>
       <c r="D107">
-        <v>1722</v>
+        <v>973</v>
       </c>
       <c r="E107">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F107" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G107" t="s">
         <v>12</v>
       </c>
       <c r="H107">
-        <v>861</v>
+        <v>973</v>
       </c>
       <c r="I107" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B108" t="s">
         <v>240</v>
       </c>
       <c r="C108">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="D108">
-        <v>973</v>
+        <v>1278</v>
       </c>
       <c r="E108">
         <v>60</v>
@@ -4586,7 +4580,7 @@
         <v>12</v>
       </c>
       <c r="H108">
-        <v>973</v>
+        <v>852</v>
       </c>
       <c r="I108" t="s">
         <v>13</v>
@@ -4594,16 +4588,16 @@
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B109" t="s">
         <v>242</v>
       </c>
       <c r="C109">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D109">
-        <v>1278</v>
+        <v>1428</v>
       </c>
       <c r="E109">
         <v>60</v>
@@ -4615,15 +4609,15 @@
         <v>12</v>
       </c>
       <c r="H109">
-        <v>852</v>
+        <v>1428</v>
       </c>
       <c r="I109" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B110" t="s">
         <v>244</v>
@@ -4632,7 +4626,7 @@
         <v>60</v>
       </c>
       <c r="D110">
-        <v>1428</v>
+        <v>1527</v>
       </c>
       <c r="E110">
         <v>60</v>
@@ -4644,24 +4638,24 @@
         <v>12</v>
       </c>
       <c r="H110">
-        <v>1428</v>
+        <v>1527</v>
       </c>
       <c r="I110" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B111" t="s">
         <v>246</v>
       </c>
       <c r="C111">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D111">
-        <v>1527</v>
+        <v>1817</v>
       </c>
       <c r="E111">
         <v>60</v>
@@ -4673,53 +4667,53 @@
         <v>12</v>
       </c>
       <c r="H111">
-        <v>1527</v>
+        <v>1090</v>
       </c>
       <c r="I111" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B112" t="s">
+        <v>240</v>
+      </c>
+      <c r="C112">
+        <v>90</v>
+      </c>
+      <c r="D112">
+        <v>1222</v>
+      </c>
+      <c r="E112">
+        <v>60</v>
+      </c>
+      <c r="F112" t="s">
         <v>248</v>
       </c>
-      <c r="C112">
-        <v>100</v>
-      </c>
-      <c r="D112">
-        <v>1817</v>
-      </c>
-      <c r="E112">
-        <v>60</v>
-      </c>
-      <c r="F112" t="s">
-        <v>249</v>
-      </c>
       <c r="G112" t="s">
         <v>12</v>
       </c>
       <c r="H112">
-        <v>1090</v>
+        <v>815</v>
       </c>
       <c r="I112" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B113" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="C113">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D113">
-        <v>1222</v>
+        <v>1587</v>
       </c>
       <c r="E113">
         <v>60</v>
@@ -4731,24 +4725,24 @@
         <v>12</v>
       </c>
       <c r="H113">
-        <v>815</v>
+        <v>1587</v>
       </c>
       <c r="I113" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B114" t="s">
         <v>251</v>
       </c>
       <c r="C114">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D114">
-        <v>1587</v>
+        <v>3667</v>
       </c>
       <c r="E114">
         <v>60</v>
@@ -4760,7 +4754,7 @@
         <v>12</v>
       </c>
       <c r="H114">
-        <v>1587</v>
+        <v>1834</v>
       </c>
       <c r="I114" t="s">
         <v>19</v>
@@ -4768,28 +4762,28 @@
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="B115" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C115">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D115">
-        <v>3667</v>
+        <v>1283</v>
       </c>
       <c r="E115">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F115" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G115" t="s">
         <v>12</v>
       </c>
       <c r="H115">
-        <v>1834</v>
+        <v>642</v>
       </c>
       <c r="I115" t="s">
         <v>19</v>
@@ -4797,16 +4791,16 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B116" t="s">
         <v>256</v>
       </c>
       <c r="C116">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="D116">
-        <v>1283</v>
+        <v>848</v>
       </c>
       <c r="E116">
         <v>30</v>
@@ -4818,24 +4812,24 @@
         <v>12</v>
       </c>
       <c r="H116">
-        <v>642</v>
+        <v>283</v>
       </c>
       <c r="I116" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B117" t="s">
         <v>258</v>
       </c>
       <c r="C117">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D117">
-        <v>848</v>
+        <v>888</v>
       </c>
       <c r="E117">
         <v>30</v>
@@ -4847,24 +4841,24 @@
         <v>12</v>
       </c>
       <c r="H117">
-        <v>283</v>
+        <v>888</v>
       </c>
       <c r="I117" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B118" t="s">
         <v>260</v>
       </c>
       <c r="C118">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="D118">
-        <v>888</v>
+        <v>409</v>
       </c>
       <c r="E118">
         <v>30</v>
@@ -4876,24 +4870,24 @@
         <v>12</v>
       </c>
       <c r="H118">
-        <v>888</v>
+        <v>102</v>
       </c>
       <c r="I118" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B119" t="s">
         <v>262</v>
       </c>
       <c r="C119">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D119">
-        <v>409</v>
+        <v>1064</v>
       </c>
       <c r="E119">
         <v>30</v>
@@ -4905,36 +4899,36 @@
         <v>12</v>
       </c>
       <c r="H119">
-        <v>102</v>
+        <v>532</v>
       </c>
       <c r="I119" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="B120" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C120">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D120">
-        <v>1064</v>
+        <v>1809</v>
       </c>
       <c r="E120">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F120" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G120" t="s">
         <v>12</v>
       </c>
       <c r="H120">
-        <v>532</v>
+        <v>904</v>
       </c>
       <c r="I120" t="s">
         <v>16</v>
@@ -4942,16 +4936,16 @@
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B121" t="s">
         <v>267</v>
       </c>
       <c r="C121">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="D121">
-        <v>1809</v>
+        <v>2333</v>
       </c>
       <c r="E121">
         <v>60</v>
@@ -4963,24 +4957,24 @@
         <v>12</v>
       </c>
       <c r="H121">
-        <v>904</v>
+        <v>1555</v>
       </c>
       <c r="I121" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B122" t="s">
         <v>269</v>
       </c>
       <c r="C122">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="D122">
-        <v>2333</v>
+        <v>1761</v>
       </c>
       <c r="E122">
         <v>60</v>
@@ -4992,24 +4986,24 @@
         <v>12</v>
       </c>
       <c r="H122">
-        <v>1555</v>
+        <v>1057</v>
       </c>
       <c r="I122" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B123" t="s">
         <v>271</v>
       </c>
       <c r="C123">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="D123">
-        <v>1761</v>
+        <v>1103</v>
       </c>
       <c r="E123">
         <v>60</v>
@@ -5021,15 +5015,15 @@
         <v>12</v>
       </c>
       <c r="H123">
-        <v>1057</v>
+        <v>552</v>
       </c>
       <c r="I123" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B124" t="s">
         <v>273</v>
@@ -5038,7 +5032,7 @@
         <v>120</v>
       </c>
       <c r="D124">
-        <v>1103</v>
+        <v>1457</v>
       </c>
       <c r="E124">
         <v>60</v>
@@ -5050,7 +5044,7 @@
         <v>12</v>
       </c>
       <c r="H124">
-        <v>552</v>
+        <v>728</v>
       </c>
       <c r="I124" t="s">
         <v>13</v>
@@ -5058,16 +5052,16 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B125" t="s">
         <v>275</v>
       </c>
       <c r="C125">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="D125">
-        <v>1457</v>
+        <v>2130</v>
       </c>
       <c r="E125">
         <v>60</v>
@@ -5079,24 +5073,24 @@
         <v>12</v>
       </c>
       <c r="H125">
-        <v>728</v>
+        <v>2556</v>
       </c>
       <c r="I125" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B126" t="s">
         <v>277</v>
       </c>
       <c r="C126">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D126">
-        <v>2130</v>
+        <v>1792</v>
       </c>
       <c r="E126">
         <v>60</v>
@@ -5108,7 +5102,7 @@
         <v>12</v>
       </c>
       <c r="H126">
-        <v>2556</v>
+        <v>1792</v>
       </c>
       <c r="I126" t="s">
         <v>19</v>
@@ -5116,45 +5110,45 @@
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B127" t="s">
+        <v>265</v>
+      </c>
+      <c r="C127">
+        <v>120</v>
+      </c>
+      <c r="D127">
+        <v>2234</v>
+      </c>
+      <c r="E127">
+        <v>60</v>
+      </c>
+      <c r="F127" t="s">
         <v>279</v>
       </c>
-      <c r="C127">
-        <v>60</v>
-      </c>
-      <c r="D127">
-        <v>1792</v>
-      </c>
-      <c r="E127">
-        <v>60</v>
-      </c>
-      <c r="F127" t="s">
-        <v>280</v>
-      </c>
       <c r="G127" t="s">
         <v>12</v>
       </c>
       <c r="H127">
-        <v>1792</v>
+        <v>1117</v>
       </c>
       <c r="I127" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B128" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
       <c r="C128">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D128">
-        <v>2234</v>
+        <v>825</v>
       </c>
       <c r="E128">
         <v>60</v>
@@ -5166,24 +5160,24 @@
         <v>12</v>
       </c>
       <c r="H128">
-        <v>1117</v>
+        <v>825</v>
       </c>
       <c r="I128" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B129" t="s">
         <v>282</v>
       </c>
       <c r="C129">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D129">
-        <v>825</v>
+        <v>750</v>
       </c>
       <c r="E129">
         <v>60</v>
@@ -5195,7 +5189,7 @@
         <v>12</v>
       </c>
       <c r="H129">
-        <v>825</v>
+        <v>375</v>
       </c>
       <c r="I129" t="s">
         <v>13</v>
@@ -5203,28 +5197,28 @@
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>266</v>
+        <v>284</v>
       </c>
       <c r="B130" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C130">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="D130">
-        <v>750</v>
+        <v>235</v>
       </c>
       <c r="E130">
         <v>60</v>
       </c>
       <c r="F130" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G130" t="s">
         <v>12</v>
       </c>
       <c r="H130">
-        <v>375</v>
+        <v>470</v>
       </c>
       <c r="I130" t="s">
         <v>13</v>
@@ -5232,7 +5226,7 @@
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B131" t="s">
         <v>287</v>
@@ -5241,7 +5235,7 @@
         <v>30</v>
       </c>
       <c r="D131">
-        <v>235</v>
+        <v>263</v>
       </c>
       <c r="E131">
         <v>60</v>
@@ -5253,24 +5247,24 @@
         <v>12</v>
       </c>
       <c r="H131">
-        <v>470</v>
+        <v>526</v>
       </c>
       <c r="I131" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B132" t="s">
         <v>289</v>
       </c>
       <c r="C132">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D132">
-        <v>263</v>
+        <v>594</v>
       </c>
       <c r="E132">
         <v>60</v>
@@ -5282,24 +5276,24 @@
         <v>12</v>
       </c>
       <c r="H132">
-        <v>526</v>
+        <v>356</v>
       </c>
       <c r="I132" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B133" t="s">
         <v>291</v>
       </c>
       <c r="C133">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D133">
-        <v>594</v>
+        <v>1024</v>
       </c>
       <c r="E133">
         <v>60</v>
@@ -5311,15 +5305,15 @@
         <v>12</v>
       </c>
       <c r="H133">
-        <v>356</v>
+        <v>683</v>
       </c>
       <c r="I133" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B134" t="s">
         <v>293</v>
@@ -5328,7 +5322,7 @@
         <v>90</v>
       </c>
       <c r="D134">
-        <v>1024</v>
+        <v>1650</v>
       </c>
       <c r="E134">
         <v>60</v>
@@ -5340,24 +5334,24 @@
         <v>12</v>
       </c>
       <c r="H134">
-        <v>683</v>
+        <v>1100</v>
       </c>
       <c r="I134" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B135" t="s">
         <v>295</v>
       </c>
       <c r="C135">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D135">
-        <v>1650</v>
+        <v>899</v>
       </c>
       <c r="E135">
         <v>60</v>
@@ -5369,7 +5363,7 @@
         <v>12</v>
       </c>
       <c r="H135">
-        <v>1100</v>
+        <v>899</v>
       </c>
       <c r="I135" t="s">
         <v>19</v>
@@ -5377,7 +5371,7 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B136" t="s">
         <v>297</v>
@@ -5386,7 +5380,7 @@
         <v>60</v>
       </c>
       <c r="D136">
-        <v>899</v>
+        <v>263</v>
       </c>
       <c r="E136">
         <v>60</v>
@@ -5398,36 +5392,36 @@
         <v>12</v>
       </c>
       <c r="H136">
-        <v>899</v>
+        <v>263</v>
       </c>
       <c r="I136" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="B137" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C137">
         <v>60</v>
       </c>
       <c r="D137">
-        <v>263</v>
+        <v>712</v>
       </c>
       <c r="E137">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F137" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G137" t="s">
         <v>12</v>
       </c>
       <c r="H137">
-        <v>263</v>
+        <v>356</v>
       </c>
       <c r="I137" t="s">
         <v>13</v>
@@ -5435,16 +5429,16 @@
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B138" t="s">
         <v>302</v>
       </c>
       <c r="C138">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D138">
-        <v>712</v>
+        <v>595</v>
       </c>
       <c r="E138">
         <v>30</v>
@@ -5456,24 +5450,24 @@
         <v>12</v>
       </c>
       <c r="H138">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="I138" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B139" t="s">
         <v>304</v>
       </c>
       <c r="C139">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="D139">
-        <v>595</v>
+        <v>385</v>
       </c>
       <c r="E139">
         <v>30</v>
@@ -5485,24 +5479,24 @@
         <v>12</v>
       </c>
       <c r="H139">
-        <v>357</v>
+        <v>96</v>
       </c>
       <c r="I139" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B140" t="s">
         <v>306</v>
       </c>
       <c r="C140">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D140">
-        <v>385</v>
+        <v>481</v>
       </c>
       <c r="E140">
         <v>30</v>
@@ -5514,7 +5508,7 @@
         <v>12</v>
       </c>
       <c r="H140">
-        <v>96</v>
+        <v>241</v>
       </c>
       <c r="I140" t="s">
         <v>13</v>
@@ -5522,7 +5516,7 @@
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B141" t="s">
         <v>308</v>
@@ -5531,7 +5525,7 @@
         <v>60</v>
       </c>
       <c r="D141">
-        <v>481</v>
+        <v>780</v>
       </c>
       <c r="E141">
         <v>30</v>
@@ -5543,15 +5537,15 @@
         <v>12</v>
       </c>
       <c r="H141">
-        <v>241</v>
+        <v>390</v>
       </c>
       <c r="I141" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B142" t="s">
         <v>310</v>
@@ -5560,7 +5554,7 @@
         <v>60</v>
       </c>
       <c r="D142">
-        <v>780</v>
+        <v>1656</v>
       </c>
       <c r="E142">
         <v>30</v>
@@ -5572,24 +5566,24 @@
         <v>12</v>
       </c>
       <c r="H142">
-        <v>390</v>
+        <v>828</v>
       </c>
       <c r="I142" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B143" t="s">
         <v>312</v>
       </c>
       <c r="C143">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D143">
-        <v>1656</v>
+        <v>901</v>
       </c>
       <c r="E143">
         <v>30</v>
@@ -5601,7 +5595,7 @@
         <v>12</v>
       </c>
       <c r="H143">
-        <v>828</v>
+        <v>901</v>
       </c>
       <c r="I143" t="s">
         <v>19</v>
@@ -5609,36 +5603,36 @@
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="B144" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C144">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D144">
-        <v>901</v>
+        <v>2566</v>
       </c>
       <c r="E144">
         <v>30</v>
       </c>
       <c r="F144" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G144" t="s">
         <v>12</v>
       </c>
       <c r="H144">
-        <v>901</v>
+        <v>1283</v>
       </c>
       <c r="I144" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B145" t="s">
         <v>317</v>
@@ -5647,7 +5641,7 @@
         <v>60</v>
       </c>
       <c r="D145">
-        <v>2566</v>
+        <v>8672</v>
       </c>
       <c r="E145">
         <v>30</v>
@@ -5659,24 +5653,24 @@
         <v>12</v>
       </c>
       <c r="H145">
-        <v>1283</v>
+        <v>4336</v>
       </c>
       <c r="I145" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B146" t="s">
         <v>319</v>
       </c>
       <c r="C146">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D146">
-        <v>8672</v>
+        <v>6418</v>
       </c>
       <c r="E146">
         <v>30</v>
@@ -5688,7 +5682,7 @@
         <v>12</v>
       </c>
       <c r="H146">
-        <v>4336</v>
+        <v>6418</v>
       </c>
       <c r="I146" t="s">
         <v>19</v>
@@ -5696,16 +5690,16 @@
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B147" t="s">
         <v>321</v>
       </c>
       <c r="C147">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D147">
-        <v>6418</v>
+        <v>4309</v>
       </c>
       <c r="E147">
         <v>30</v>
@@ -5717,24 +5711,24 @@
         <v>12</v>
       </c>
       <c r="H147">
-        <v>6418</v>
+        <v>2154</v>
       </c>
       <c r="I147" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B148" t="s">
         <v>323</v>
       </c>
       <c r="C148">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D148">
-        <v>4309</v>
+        <v>605</v>
       </c>
       <c r="E148">
         <v>30</v>
@@ -5746,24 +5740,24 @@
         <v>12</v>
       </c>
       <c r="H148">
-        <v>2154</v>
+        <v>182</v>
       </c>
       <c r="I148" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B149" t="s">
         <v>325</v>
       </c>
       <c r="C149">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D149">
-        <v>605</v>
+        <v>2520</v>
       </c>
       <c r="E149">
         <v>30</v>
@@ -5775,7 +5769,7 @@
         <v>12</v>
       </c>
       <c r="H149">
-        <v>182</v>
+        <v>1260</v>
       </c>
       <c r="I149" t="s">
         <v>13</v>
@@ -5783,7 +5777,7 @@
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B150" t="s">
         <v>327</v>
@@ -5792,7 +5786,7 @@
         <v>60</v>
       </c>
       <c r="D150">
-        <v>2520</v>
+        <v>5379</v>
       </c>
       <c r="E150">
         <v>30</v>
@@ -5804,15 +5798,15 @@
         <v>12</v>
       </c>
       <c r="H150">
-        <v>1260</v>
+        <v>2690</v>
       </c>
       <c r="I150" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B151" t="s">
         <v>329</v>
@@ -5821,7 +5815,7 @@
         <v>60</v>
       </c>
       <c r="D151">
-        <v>5379</v>
+        <v>2103</v>
       </c>
       <c r="E151">
         <v>30</v>
@@ -5833,36 +5827,36 @@
         <v>12</v>
       </c>
       <c r="H151">
-        <v>2690</v>
+        <v>1052</v>
       </c>
       <c r="I151" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>316</v>
+        <v>331</v>
       </c>
       <c r="B152" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C152">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D152">
-        <v>2103</v>
+        <v>1026</v>
       </c>
       <c r="E152">
         <v>30</v>
       </c>
       <c r="F152" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G152" t="s">
         <v>12</v>
       </c>
       <c r="H152">
-        <v>1052</v>
+        <v>308</v>
       </c>
       <c r="I152" t="s">
         <v>13</v>
@@ -5870,16 +5864,16 @@
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B153" t="s">
         <v>334</v>
       </c>
       <c r="C153">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D153">
-        <v>1026</v>
+        <v>961</v>
       </c>
       <c r="E153">
         <v>30</v>
@@ -5891,53 +5885,53 @@
         <v>12</v>
       </c>
       <c r="H153">
-        <v>308</v>
+        <v>480</v>
       </c>
       <c r="I153" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B154" t="s">
+        <v>332</v>
+      </c>
+      <c r="C154">
+        <v>100</v>
+      </c>
+      <c r="D154">
+        <v>1046</v>
+      </c>
+      <c r="E154">
+        <v>30</v>
+      </c>
+      <c r="F154" t="s">
         <v>336</v>
       </c>
-      <c r="C154">
-        <v>60</v>
-      </c>
-      <c r="D154">
-        <v>961</v>
-      </c>
-      <c r="E154">
-        <v>30</v>
-      </c>
-      <c r="F154" t="s">
-        <v>337</v>
-      </c>
       <c r="G154" t="s">
         <v>12</v>
       </c>
       <c r="H154">
-        <v>480</v>
+        <v>314</v>
       </c>
       <c r="I154" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B155" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C155">
         <v>100</v>
       </c>
       <c r="D155">
-        <v>1046</v>
+        <v>2455</v>
       </c>
       <c r="E155">
         <v>30</v>
@@ -5949,15 +5943,15 @@
         <v>12</v>
       </c>
       <c r="H155">
-        <v>314</v>
+        <v>736</v>
       </c>
       <c r="I155" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B156" t="s">
         <v>339</v>
@@ -5966,7 +5960,7 @@
         <v>100</v>
       </c>
       <c r="D156">
-        <v>2455</v>
+        <v>473</v>
       </c>
       <c r="E156">
         <v>30</v>
@@ -5978,24 +5972,24 @@
         <v>12</v>
       </c>
       <c r="H156">
-        <v>736</v>
+        <v>142</v>
       </c>
       <c r="I156" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B157" t="s">
         <v>341</v>
       </c>
       <c r="C157">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D157">
-        <v>473</v>
+        <v>727</v>
       </c>
       <c r="E157">
         <v>30</v>
@@ -6007,53 +6001,50 @@
         <v>12</v>
       </c>
       <c r="H157">
-        <v>142</v>
+        <v>364</v>
       </c>
       <c r="I157" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="B158" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C158">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="D158">
-        <v>727</v>
+        <v>640</v>
       </c>
       <c r="E158">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="F158" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G158" t="s">
         <v>12</v>
       </c>
       <c r="H158">
-        <v>364</v>
-      </c>
-      <c r="I158" t="s">
-        <v>16</v>
+        <v>480</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B159" t="s">
         <v>346</v>
       </c>
       <c r="C159">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D159">
-        <v>640</v>
+        <v>1411</v>
       </c>
       <c r="E159">
         <v>150</v>
@@ -6065,21 +6056,21 @@
         <v>12</v>
       </c>
       <c r="H159">
-        <v>480</v>
+        <v>423</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B160" t="s">
         <v>348</v>
       </c>
       <c r="C160">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D160">
-        <v>1411</v>
+        <v>660</v>
       </c>
       <c r="E160">
         <v>150</v>
@@ -6091,12 +6082,12 @@
         <v>12</v>
       </c>
       <c r="H160">
-        <v>423</v>
+        <v>495</v>
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B161" t="s">
         <v>350</v>
@@ -6122,7 +6113,7 @@
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B162" t="s">
         <v>352</v>
@@ -6131,7 +6122,7 @@
         <v>200</v>
       </c>
       <c r="D162">
-        <v>660</v>
+        <v>845</v>
       </c>
       <c r="E162">
         <v>150</v>
@@ -6143,12 +6134,12 @@
         <v>12</v>
       </c>
       <c r="H162">
-        <v>495</v>
+        <v>634</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B163" t="s">
         <v>354</v>
@@ -6157,7 +6148,7 @@
         <v>200</v>
       </c>
       <c r="D163">
-        <v>845</v>
+        <v>563</v>
       </c>
       <c r="E163">
         <v>150</v>
@@ -6169,21 +6160,21 @@
         <v>12</v>
       </c>
       <c r="H163">
-        <v>634</v>
+        <v>422</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B164" t="s">
         <v>356</v>
       </c>
       <c r="C164">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D164">
-        <v>563</v>
+        <v>1525</v>
       </c>
       <c r="E164">
         <v>150</v>
@@ -6195,12 +6186,12 @@
         <v>12</v>
       </c>
       <c r="H164">
-        <v>422</v>
+        <v>458</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B165" t="s">
         <v>358</v>
@@ -6209,7 +6200,7 @@
         <v>500</v>
       </c>
       <c r="D165">
-        <v>1525</v>
+        <v>1490</v>
       </c>
       <c r="E165">
         <v>150</v>
@@ -6221,21 +6212,21 @@
         <v>12</v>
       </c>
       <c r="H165">
-        <v>458</v>
+        <v>447</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B166" t="s">
         <v>360</v>
       </c>
       <c r="C166">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="D166">
-        <v>1490</v>
+        <v>385</v>
       </c>
       <c r="E166">
         <v>150</v>
@@ -6247,21 +6238,21 @@
         <v>12</v>
       </c>
       <c r="H166">
-        <v>447</v>
+        <v>193</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B167" t="s">
         <v>362</v>
       </c>
       <c r="C167">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D167">
-        <v>385</v>
+        <v>668</v>
       </c>
       <c r="E167">
         <v>150</v>
@@ -6273,32 +6264,6 @@
         <v>12</v>
       </c>
       <c r="H167">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
-        <v>345</v>
-      </c>
-      <c r="B168" t="s">
-        <v>364</v>
-      </c>
-      <c r="C168">
-        <v>200</v>
-      </c>
-      <c r="D168">
-        <v>668</v>
-      </c>
-      <c r="E168">
-        <v>150</v>
-      </c>
-      <c r="F168" t="s">
-        <v>365</v>
-      </c>
-      <c r="G168" t="s">
-        <v>12</v>
-      </c>
-      <c r="H168">
         <v>501</v>
       </c>
     </row>

</xml_diff>